<commit_message>
add json_file generate .py files
</commit_message>
<xml_diff>
--- a/example_output/spreadsheets/indirect_costs.xlsx
+++ b/example_output/spreadsheets/indirect_costs.xlsx
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jan-15</t>
+          <t>Jan-16</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -477,7 +477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Feb-15</t>
+          <t>Feb-16</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -496,7 +496,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mar-15</t>
+          <t>Mar-16</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -515,7 +515,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Apr-15</t>
+          <t>Apr-16</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -534,7 +534,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>May-15</t>
+          <t>May-16</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -553,7 +553,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jun-15</t>
+          <t>Jun-16</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -572,7 +572,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jul-15</t>
+          <t>Jul-16</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -591,7 +591,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aug-15</t>
+          <t>Aug-16</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -610,7 +610,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sep-15</t>
+          <t>Sep-16</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -629,7 +629,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Oct-15</t>
+          <t>Oct-16</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -648,7 +648,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nov-15</t>
+          <t>Nov-16</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -667,7 +667,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dec-15</t>
+          <t>Dec-16</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -686,7 +686,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jan-16</t>
+          <t>Jan-17</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -705,7 +705,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Feb-16</t>
+          <t>Feb-17</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -724,7 +724,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mar-16</t>
+          <t>Mar-17</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -743,7 +743,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Apr-16</t>
+          <t>Apr-17</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -762,7 +762,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>May-16</t>
+          <t>May-17</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -781,7 +781,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jun-16</t>
+          <t>Jun-17</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -800,7 +800,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jul-16</t>
+          <t>Jul-17</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -819,7 +819,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aug-16</t>
+          <t>Aug-17</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -838,7 +838,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sep-16</t>
+          <t>Sep-17</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -857,7 +857,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Oct-16</t>
+          <t>Oct-17</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -876,7 +876,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Nov-16</t>
+          <t>Nov-17</t>
         </is>
       </c>
       <c r="B24" t="n">

</xml_diff>

<commit_message>
enabling passing time intervals
</commit_message>
<xml_diff>
--- a/example_output/spreadsheets/indirect_costs.xlsx
+++ b/example_output/spreadsheets/indirect_costs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jan-15</t>
+          <t>Jan-20</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -477,7 +477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Feb-15</t>
+          <t>Feb-20</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -496,7 +496,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mar-15</t>
+          <t>Mar-20</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -515,7 +515,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Apr-15</t>
+          <t>Apr-20</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -534,7 +534,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>May-15</t>
+          <t>May-20</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -553,7 +553,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jun-15</t>
+          <t>Jun-20</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -572,7 +572,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jul-15</t>
+          <t>Jul-20</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -591,7 +591,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aug-15</t>
+          <t>Aug-20</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -610,7 +610,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sep-15</t>
+          <t>Sep-20</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -629,7 +629,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Oct-15</t>
+          <t>Oct-20</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -648,7 +648,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nov-15</t>
+          <t>Nov-20</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -662,234 +662,6 @@
       </c>
       <c r="E12" t="n">
         <v>321210.78</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Dec-15</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" t="n">
-        <v>258650.74</v>
-      </c>
-      <c r="D13" t="n">
-        <v>55717.72</v>
-      </c>
-      <c r="E13" t="n">
-        <v>314368.46</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Jan-16</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" t="n">
-        <v>252175.98</v>
-      </c>
-      <c r="D14" t="n">
-        <v>58329.03</v>
-      </c>
-      <c r="E14" t="n">
-        <v>310505.01</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Feb-16</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="C15" t="n">
-        <v>244305.23</v>
-      </c>
-      <c r="D15" t="n">
-        <v>60012.48</v>
-      </c>
-      <c r="E15" t="n">
-        <v>304317.71</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Mar-16</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" t="n">
-        <v>241621.2</v>
-      </c>
-      <c r="D16" t="n">
-        <v>58528.24</v>
-      </c>
-      <c r="E16" t="n">
-        <v>300149.44</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Apr-16</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>239032.88</v>
-      </c>
-      <c r="D17" t="n">
-        <v>63694.36</v>
-      </c>
-      <c r="E17" t="n">
-        <v>302727.24</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>May-16</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" t="n">
-        <v>239635.18</v>
-      </c>
-      <c r="D18" t="n">
-        <v>57655.44</v>
-      </c>
-      <c r="E18" t="n">
-        <v>297290.62</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Jun-16</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
-        <v>243293.68</v>
-      </c>
-      <c r="D19" t="n">
-        <v>54036.96</v>
-      </c>
-      <c r="E19" t="n">
-        <v>297330.64</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Jul-16</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="n">
-        <v>242000.98</v>
-      </c>
-      <c r="D20" t="n">
-        <v>50080.31</v>
-      </c>
-      <c r="E20" t="n">
-        <v>292081.29</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Aug-16</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>234265.6</v>
-      </c>
-      <c r="D21" t="n">
-        <v>54302.69</v>
-      </c>
-      <c r="E21" t="n">
-        <v>288568.29</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Sep-16</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>240823.88</v>
-      </c>
-      <c r="D22" t="n">
-        <v>56481.26</v>
-      </c>
-      <c r="E22" t="n">
-        <v>297305.14</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Oct-16</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" t="n">
-        <v>240985.37</v>
-      </c>
-      <c r="D23" t="n">
-        <v>56440.75</v>
-      </c>
-      <c r="E23" t="n">
-        <v>297426.12</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Nov-16</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" t="n">
-        <v>235683.88</v>
-      </c>
-      <c r="D24" t="n">
-        <v>55490.59</v>
-      </c>
-      <c r="E24" t="n">
-        <v>291174.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added func for excel versions; Modified date col
</commit_message>
<xml_diff>
--- a/example_output/spreadsheets/indirect_costs.xlsx
+++ b/example_output/spreadsheets/indirect_costs.xlsx
@@ -431,7 +431,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Month</t>
+          <t>YearMonth</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jan-20</t>
+          <t>2020-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -477,7 +477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Feb-20</t>
+          <t>2020-02</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -496,7 +496,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mar-20</t>
+          <t>2020-03</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -515,7 +515,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Apr-20</t>
+          <t>2020-04</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -534,7 +534,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>May-20</t>
+          <t>2020-05</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -553,7 +553,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jun-20</t>
+          <t>2020-06</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -572,7 +572,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jul-20</t>
+          <t>2020-07</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -591,7 +591,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aug-20</t>
+          <t>2020-08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -610,7 +610,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sep-20</t>
+          <t>2020-09</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -629,7 +629,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Oct-20</t>
+          <t>2020-10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -648,7 +648,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nov-20</t>
+          <t>2020-11</t>
         </is>
       </c>
       <c r="B12" t="n">

</xml_diff>

<commit_message>
upload json and ss to gcp
</commit_message>
<xml_diff>
--- a/example_output/spreadsheets/indirect_costs.xlsx
+++ b/example_output/spreadsheets/indirect_costs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>